<commit_message>
feat: add inventory management and configuration tests
- Implemented the main inventory component with navigation for different screens.
- Created end-to-end tests for complete process configuration, including setting up a new process, importing data, and finalizing the configuration.
- Added tests for handling test data, including importing inventory and economic data, calculating values, and generating reports.
- Included functionality to delete processes without inventory and ensure demonstration processes are handled correctly.
- Established a test for initiating a process from a filled PL-01 format, ensuring data is imported correctly.
</commit_message>
<xml_diff>
--- a/datos_de_prueba/02_caso_con_problemas/PL-03_toma_inventario_fisico.xlsx
+++ b/datos_de_prueba/02_caso_con_problemas/PL-03_toma_inventario_fisico.xlsx
@@ -455,13 +455,13 @@
     <t>166002092</t>
   </si>
   <si>
-    <t>EQUIPO CONTADO DESPUES DEL CORTE</t>
+    <t>EQUIPO CON TOMA EN EL FUTURO</t>
   </si>
   <si>
     <t>SN-X9</t>
   </si>
   <si>
-    <t>2026-02-14</t>
+    <t>2030-02-14</t>
   </si>
 </sst>
 </file>

</xml_diff>